<commit_message>
Phase A.3: 제외 사이트 3개 복구 — 총 41개 사이트 (HTML 34 + CCEI 7)
인천테크노파크(POST 페이지네이션+세션), 건국대학교(K2Web SSO 통과),
대전기업정보포털(사업공고 사실상 입찰) 추가. generic_scraper에 POST
페이지네이션, 세션 초기화, JS 링크 변환 기능 추가.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/work_log2/site_verification.xlsx
+++ b/work_log2/site_verification.xlsx
@@ -574,7 +574,7 @@
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Phase A.3 스크래핑 대상 사이트 검증 결과 (2026-03-30 최종)</t>
+          <t>Phase A.3 스크래핑 대상 사이트 검증 결과 (2026-03-30 최종 업데이트)</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>✅ 구현 완료 — HTML 스크래핑 (31개)</t>
+          <t>✅ 구현 완료 — HTML 스크래핑 (34개)</t>
         </is>
       </c>
       <c r="B3" s="4" t="n"/>
@@ -1267,79 +1267,79 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>✅ 구현 완료 — CCEI 입찰공고 JSON API (7개)</t>
-        </is>
-      </c>
-      <c r="B35" s="10" t="n"/>
-      <c r="C35" s="10" t="n"/>
-      <c r="D35" s="10" t="n"/>
-      <c r="E35" s="10" t="n"/>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="5" t="inlineStr"/>
+      <c r="B35" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>인천테크노파크</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>https://www.itp.or.kr/intro.asp?tmid=14</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>POST 페이지네이션 + 세션 쿠키</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="5" t="inlineStr"/>
       <c r="B36" s="6" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>CCEI-경기</t>
+          <t>건국대학교</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/gyeonggi/allim/allimList.json</t>
+          <t>https://www.konkuk.ac.kr/konkuk/2243/subview.do</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>POST JSON API</t>
+          <t>K2Web CMS, SSO 통과 후 접근 가능</t>
         </is>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="5" t="inlineStr"/>
       <c r="B37" s="6" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>CCEI-경남</t>
+          <t>대전기업정보포털</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/gyeongnam/allim/allimList.json</t>
+          <t>https://www.dips.or.kr/pbanc?mid=a10201000000</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>POST JSON API</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="5" t="inlineStr"/>
-      <c r="B38" s="6" t="n">
-        <v>34</v>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>CCEI-대구</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>https://ccei.creativekorea.or.kr/daegu/allim/allimList.json</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
-        <is>
-          <t>POST JSON API</t>
-        </is>
-      </c>
+          <t>사업공고 (사실상 입찰), PDF 링크</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>✅ 구현 완료 — CCEI 입찰공고 JSON API (7개)</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="n"/>
+      <c r="C38" s="10" t="n"/>
+      <c r="D38" s="10" t="n"/>
+      <c r="E38" s="10" t="n"/>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="5" t="inlineStr"/>
@@ -1348,12 +1348,12 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>CCEI-부산</t>
+          <t>CCEI-경기</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/busan/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/gyeonggi/allim/allimList.json</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
@@ -1369,12 +1369,12 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>CCEI-세종</t>
+          <t>CCEI-경남</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/sejong/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/gyeongnam/allim/allimList.json</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
@@ -1390,12 +1390,12 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>CCEI-인천</t>
+          <t>CCEI-대구</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/incheon/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/daegu/allim/allimList.json</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -1411,12 +1411,12 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>CCEI-충북</t>
+          <t>CCEI-부산</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/chungbuk/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/busan/allim/allimList.json</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
@@ -1425,79 +1425,79 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="28" customHeight="1">
-      <c r="A43" s="11" t="inlineStr">
-        <is>
-          <t>🔧 추가 조치 필요 (4개)</t>
-        </is>
-      </c>
-      <c r="B43" s="12" t="n"/>
-      <c r="C43" s="12" t="n"/>
-      <c r="D43" s="12" t="n"/>
-      <c r="E43" s="12" t="n"/>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="5" t="inlineStr"/>
+      <c r="B43" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>CCEI-세종</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>https://ccei.creativekorea.or.kr/sejong/allim/allimList.json</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>POST JSON API</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="5" t="inlineStr"/>
       <c r="B44" s="6" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>경남테크노파크</t>
+          <t>CCEI-인천</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>https://www.gntp.or.kr</t>
+          <t>https://ccei.creativekorea.or.kr/incheon/allim/allimList.json</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>URL변경 필요 (원래 more.co.kr 서버 다운)</t>
+          <t>POST JSON API</t>
         </is>
       </c>
     </row>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="5" t="inlineStr"/>
       <c r="B45" s="6" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>대전정보문화산업진흥원</t>
+          <t>CCEI-충북</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>https://www.dicia.or.kr/sub.do?menuIdx=MENU_000000000000100</t>
+          <t>https://ccei.creativekorea.or.kr/chungbuk/allim/allimList.json</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>SSL 인증서 오류 — verify=False 필요</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="5" t="inlineStr"/>
-      <c r="B46" s="6" t="n">
-        <v>41</v>
-      </c>
-      <c r="C46" s="7" t="inlineStr">
-        <is>
-          <t>전주정보문화산업진흥원</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>https://www.jica.or.kr/2025/inner.php?sMenu=A4000</t>
-        </is>
-      </c>
-      <c r="E46" s="7" t="inlineStr">
-        <is>
-          <t>SSL 오류 + URL /2016/→/2025/ 변경</t>
-        </is>
-      </c>
+          <t>POST JSON API</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="28" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>🔧 추가 조치 필요 (4개)</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="n"/>
+      <c r="C46" s="12" t="n"/>
+      <c r="D46" s="12" t="n"/>
+      <c r="E46" s="12" t="n"/>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="5" t="inlineStr"/>
@@ -1506,178 +1506,178 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>한국예탁결제원</t>
+          <t>경남테크노파크</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>https://www.ksd.or.kr/ko/about-ksd/ksd-news/bid-notice</t>
+          <t>https://www.gntp.or.kr</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>React SPA — headless browser 필요</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="28" customHeight="1">
-      <c r="A48" s="13" t="inlineStr">
-        <is>
-          <t>🔄 URL 변경 필요 (2개)</t>
-        </is>
-      </c>
-      <c r="B48" s="14" t="n"/>
-      <c r="C48" s="14" t="n"/>
-      <c r="D48" s="14" t="n"/>
-      <c r="E48" s="14" t="n"/>
+          <t>URL변경 필요 (원래 more.co.kr 서버 다운)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="5" t="inlineStr"/>
+      <c r="B48" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>대전정보문화산업진흥원</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>https://www.dicia.or.kr/sub.do?menuIdx=MENU_000000000000100</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>SSL 인증서 오류 — verify=False 필요</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="5" t="inlineStr"/>
       <c r="B49" s="6" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>제주콘텐츠진흥원</t>
+          <t>전주정보문화산업진흥원</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>https://ofjeju.kr/communication/account/bid.htm</t>
+          <t>https://www.jica.or.kr/2025/inner.php?sMenu=A4000</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>기존 URL은 공지사항 → 입찰 URL로 변경</t>
+          <t>SSL 오류 + URL /2016/→/2025/ 변경</t>
         </is>
       </c>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="5" t="inlineStr"/>
       <c r="B50" s="6" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>소상공인시장진흥공단</t>
+          <t>한국예탁결제원</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
         <is>
-          <t>https://semas.or.kr/web/board/webBoardList.kmdc?bCd=220&amp;pNm=BOA0102</t>
+          <t>https://www.ksd.or.kr/ko/about-ksd/ksd-news/bid-notice</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>입찰정보 5건뿐, 실효성 낮음</t>
+          <t>React SPA — headless browser 필요</t>
         </is>
       </c>
     </row>
     <row r="51" ht="28" customHeight="1">
-      <c r="A51" s="15" t="inlineStr">
-        <is>
-          <t>🔧 JS 렌더링 보류 (1개)</t>
-        </is>
-      </c>
-      <c r="B51" s="16" t="n"/>
-      <c r="C51" s="16" t="n"/>
-      <c r="D51" s="16" t="n"/>
-      <c r="E51" s="16" t="n"/>
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>🔄 URL 변경 필요 (2개)</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="n"/>
+      <c r="C51" s="14" t="n"/>
+      <c r="D51" s="14" t="n"/>
+      <c r="E51" s="14" t="n"/>
     </row>
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="5" t="inlineStr"/>
       <c r="B52" s="6" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>한국지식재산보호원</t>
+          <t>제주콘텐츠진흥원</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
         <is>
-          <t>https://www.koipa.re.kr/home/board/brdList.do?menu_cd=000042</t>
+          <t>https://ofjeju.kr/communication/account/bid.htm</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>JS 렌더링 — BeautifulSoup 불가, API 또는 Selenium 필요</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="28" customHeight="1">
-      <c r="A53" s="17" t="inlineStr">
-        <is>
-          <t>❌ 제외 (4개)</t>
-        </is>
-      </c>
-      <c r="B53" s="18" t="n"/>
-      <c r="C53" s="18" t="n"/>
-      <c r="D53" s="18" t="n"/>
-      <c r="E53" s="18" t="n"/>
-    </row>
-    <row r="54" ht="22" customHeight="1">
-      <c r="A54" s="5" t="inlineStr"/>
-      <c r="B54" s="6" t="n">
-        <v>46</v>
-      </c>
-      <c r="C54" s="7" t="inlineStr">
-        <is>
-          <t>대전기업정보포털</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>https://www.dips.or.kr/pbanc?nPage=1&amp;mid=a10201000000</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="inlineStr">
-        <is>
-          <t>지원사업 공고, 입찰 아님</t>
-        </is>
-      </c>
+          <t>기존 URL은 공지사항 → 입찰 URL로 변경</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="5" t="inlineStr"/>
+      <c r="B53" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>소상공인시장진흥공단</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>https://semas.or.kr/web/board/webBoardList.kmdc?bCd=220&amp;pNm=BOA0102</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>입찰정보 5건뿐, 실효성 낮음</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="28" customHeight="1">
+      <c r="A54" s="15" t="inlineStr">
+        <is>
+          <t>🔧 JS 렌더링 보류 (1개)</t>
+        </is>
+      </c>
+      <c r="B54" s="16" t="n"/>
+      <c r="C54" s="16" t="n"/>
+      <c r="D54" s="16" t="n"/>
+      <c r="E54" s="16" t="n"/>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="5" t="inlineStr"/>
       <c r="B55" s="6" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>부산창업포탈</t>
+          <t>한국지식재산보호원</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>https://busanstartup.kr/biz_sup?mcode=biz02&amp;deleteYn=N&amp;busi_code=820</t>
+          <t>https://www.koipa.re.kr/home/board/brdList.do?menu_cd=000042</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>창업지원 프로그램, 입찰 아님</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="5" t="inlineStr"/>
-      <c r="B56" s="6" t="n">
-        <v>48</v>
-      </c>
-      <c r="C56" s="7" t="inlineStr">
-        <is>
-          <t>건국대학교</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>https://www.konkuk.ac.kr/konkuk/2243/subview.do</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="inlineStr">
-        <is>
-          <t>SSO 로그인 필수, 외부 스크래핑 불가</t>
-        </is>
-      </c>
+          <t>JS 렌더링 — BeautifulSoup 불가, API 또는 Selenium 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="28" customHeight="1">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>❌ 제외 (1개)</t>
+        </is>
+      </c>
+      <c r="B56" s="18" t="n"/>
+      <c r="C56" s="18" t="n"/>
+      <c r="D56" s="18" t="n"/>
+      <c r="E56" s="18" t="n"/>
     </row>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="5" t="inlineStr"/>
@@ -1686,36 +1686,36 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>인천테크노파크</t>
+          <t>부산창업포탈</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>https://www.itp.or.kr/intro.asp?tmid=14</t>
+          <t>https://busanstartup.kr/biz_sup?mcode=biz02&amp;deleteYn=N&amp;busi_code=820</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>사이트 전체 다운 (404)</t>
+          <t>창업지원 프로그램, 입찰 아님</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="19" t="inlineStr">
         <is>
-          <t>※ 구현 완료 38개 사이트는 일괄 수집 버튼 1개로 수집 가능</t>
+          <t>※ 구현 완료 41개 사이트는 일괄 수집 버튼 1개로 수집 가능</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="A35:E35"/>
     <mergeCell ref="A59:E59"/>
-    <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A54:E54"/>
     <mergeCell ref="A51:E51"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A56:E56"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <hyperlinks>
@@ -1750,23 +1750,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Phase A.3: 경남테크노파크 추가 — 총 42개 사이트 (HTML 35 + CCEI 7)
경남TP 신규 URL(gntp.or.kr) JSON POST API + grid_selector 파싱 구현.
generic_scraper에 post_json, grid_selector 기능 추가 및
빈 dict post_data falsy 버그 수정 (use_post 플래그 도입).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/work_log2/site_verification.xlsx
+++ b/work_log2/site_verification.xlsx
@@ -608,7 +608,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>✅ 구현 완료 — HTML 스크래핑 (34개)</t>
+          <t>✅ 구현 완료 — HTML 스크래핑 (35개)</t>
         </is>
       </c>
       <c r="B3" s="4" t="n"/>
@@ -1330,37 +1330,37 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="9" t="inlineStr">
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="5" t="inlineStr"/>
+      <c r="B38" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>경남테크노파크</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>https://www.gntp.or.kr/biz/apply</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>JSON POST API + grid_selector 파싱</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>✅ 구현 완료 — CCEI 입찰공고 JSON API (7개)</t>
         </is>
       </c>
-      <c r="B38" s="10" t="n"/>
-      <c r="C38" s="10" t="n"/>
-      <c r="D38" s="10" t="n"/>
-      <c r="E38" s="10" t="n"/>
-    </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="5" t="inlineStr"/>
-      <c r="B39" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>CCEI-경기</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>https://ccei.creativekorea.or.kr/gyeonggi/allim/allimList.json</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>POST JSON API</t>
-        </is>
-      </c>
+      <c r="B39" s="10" t="n"/>
+      <c r="C39" s="10" t="n"/>
+      <c r="D39" s="10" t="n"/>
+      <c r="E39" s="10" t="n"/>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="5" t="inlineStr"/>
@@ -1369,12 +1369,12 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>CCEI-경남</t>
+          <t>CCEI-경기</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/gyeongnam/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/gyeonggi/allim/allimList.json</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
@@ -1390,12 +1390,12 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>CCEI-대구</t>
+          <t>CCEI-경남</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/daegu/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/gyeongnam/allim/allimList.json</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -1411,12 +1411,12 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>CCEI-부산</t>
+          <t>CCEI-대구</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/busan/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/daegu/allim/allimList.json</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
@@ -1432,12 +1432,12 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>CCEI-세종</t>
+          <t>CCEI-부산</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/sejong/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/busan/allim/allimList.json</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
@@ -1453,12 +1453,12 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>CCEI-인천</t>
+          <t>CCEI-세종</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/incheon/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/sejong/allim/allimList.json</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
@@ -1474,51 +1474,51 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
+          <t>CCEI-인천</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>https://ccei.creativekorea.or.kr/incheon/allim/allimList.json</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>POST JSON API</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="5" t="inlineStr"/>
+      <c r="B46" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
           <t>CCEI-충북</t>
         </is>
       </c>
-      <c r="D45" s="8" t="inlineStr">
+      <c r="D46" s="8" t="inlineStr">
         <is>
           <t>https://ccei.creativekorea.or.kr/chungbuk/allim/allimList.json</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
+      <c r="E46" s="7" t="inlineStr">
         <is>
           <t>POST JSON API</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="28" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
-        <is>
-          <t>🔧 추가 조치 필요 (4개)</t>
-        </is>
-      </c>
-      <c r="B46" s="12" t="n"/>
-      <c r="C46" s="12" t="n"/>
-      <c r="D46" s="12" t="n"/>
-      <c r="E46" s="12" t="n"/>
-    </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="5" t="inlineStr"/>
-      <c r="B47" s="6" t="n">
-        <v>42</v>
-      </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>경남테크노파크</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>https://www.gntp.or.kr</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>URL변경 필요 (원래 more.co.kr 서버 다운)</t>
-        </is>
-      </c>
+    <row r="47" ht="28" customHeight="1">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>🔧 추가 조치 필요 (3개)</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="n"/>
+      <c r="C47" s="12" t="n"/>
+      <c r="D47" s="12" t="n"/>
+      <c r="E47" s="12" t="n"/>
     </row>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="5" t="inlineStr"/>
@@ -1650,7 +1650,7 @@
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="5" t="inlineStr"/>
       <c r="B55" s="6" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
@@ -1682,7 +1682,7 @@
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="5" t="inlineStr"/>
       <c r="B57" s="6" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
@@ -1703,18 +1703,18 @@
     <row r="59">
       <c r="A59" s="19" t="inlineStr">
         <is>
-          <t>※ 구현 완료 41개 사이트는 일괄 수집 버튼 1개로 수집 가능</t>
+          <t>※ 구현 완료 42개 사이트는 일괄 수집 버튼 1개로 수집 가능</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A39:E39"/>
     <mergeCell ref="A59:E59"/>
-    <mergeCell ref="A38:E38"/>
     <mergeCell ref="A54:E54"/>
     <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A47:E47"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A46:E46"/>
     <mergeCell ref="A56:E56"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
@@ -1753,14 +1753,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId45"/>

</xml_diff>

<commit_message>
Phase A.3: 추가 조치 3개 완료 — 총 46개 사이트 (HTML 38 + CCEI 7 + KSD 1)
대전정보문화(SSL verify=False), 전주정보문화(URL 변경+SSL),
한국예탁결제원(React SPA → JSON API /ko/api/content 직접 호출) 추가.
scrape_ksd() 전용 함수 구현.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/work_log2/site_verification.xlsx
+++ b/work_log2/site_verification.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,12 +60,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="009C6500"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="00974706"/>
       <sz val="11"/>
     </font>
@@ -88,7 +82,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -108,11 +102,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00B7DEE8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -157,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -191,11 +180,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -608,7 +593,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>✅ 구현 완료 — HTML 스크래핑 (36개)</t>
+          <t>✅ 구현 완료 — HTML 스크래핑 (38개)</t>
         </is>
       </c>
       <c r="B3" s="4" t="n"/>
@@ -1372,58 +1357,58 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="28" customHeight="1">
-      <c r="A40" s="9" t="inlineStr">
-        <is>
-          <t>✅ 구현 완료 — CCEI 입찰공고 JSON API (7개)</t>
-        </is>
-      </c>
-      <c r="B40" s="10" t="n"/>
-      <c r="C40" s="10" t="n"/>
-      <c r="D40" s="10" t="n"/>
-      <c r="E40" s="10" t="n"/>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="5" t="inlineStr"/>
+      <c r="B40" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>대전정보문화산업진흥원</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>https://www.dicia.or.kr/sub.do?menuIdx=MENU_000000000000100</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>SSL verify=False, board.es 구조</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="5" t="inlineStr"/>
       <c r="B41" s="6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>CCEI-경기</t>
+          <t>전주정보문화산업진흥원</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/gyeonggi/allim/allimList.json</t>
+          <t>https://www.jica.or.kr/2025/inner.php?sMenu=A4000</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>POST JSON API</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="5" t="inlineStr"/>
-      <c r="B42" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>CCEI-경남</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>https://ccei.creativekorea.or.kr/gyeongnam/allim/allimList.json</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>POST JSON API</t>
-        </is>
-      </c>
+          <t>SSL verify=False, URL /2016/→/2025/ 변경</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>✅ 구현 완료 — CCEI 입찰공고 JSON API (7개)</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="n"/>
+      <c r="C42" s="10" t="n"/>
+      <c r="D42" s="10" t="n"/>
+      <c r="E42" s="10" t="n"/>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="5" t="inlineStr"/>
@@ -1432,12 +1417,12 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>CCEI-대구</t>
+          <t>CCEI-경기</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/daegu/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/gyeonggi/allim/allimList.json</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
@@ -1453,12 +1438,12 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>CCEI-부산</t>
+          <t>CCEI-경남</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/busan/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/gyeongnam/allim/allimList.json</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
@@ -1474,12 +1459,12 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>CCEI-세종</t>
+          <t>CCEI-대구</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/sejong/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/daegu/allim/allimList.json</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -1495,12 +1480,12 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>CCEI-인천</t>
+          <t>CCEI-부산</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/incheon/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/busan/allim/allimList.json</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -1516,12 +1501,12 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>CCEI-충북</t>
+          <t>CCEI-세종</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/chungbuk/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/sejong/allim/allimList.json</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
@@ -1530,58 +1515,58 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="28" customHeight="1">
-      <c r="A48" s="11" t="inlineStr">
-        <is>
-          <t>🔧 추가 조치 필요 (3개)</t>
-        </is>
-      </c>
-      <c r="B48" s="12" t="n"/>
-      <c r="C48" s="12" t="n"/>
-      <c r="D48" s="12" t="n"/>
-      <c r="E48" s="12" t="n"/>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="5" t="inlineStr"/>
+      <c r="B48" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>CCEI-인천</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>https://ccei.creativekorea.or.kr/incheon/allim/allimList.json</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>POST JSON API</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="5" t="inlineStr"/>
       <c r="B49" s="6" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>대전정보문화산업진흥원</t>
+          <t>CCEI-충북</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>https://www.dicia.or.kr/sub.do?menuIdx=MENU_000000000000100</t>
+          <t>https://ccei.creativekorea.or.kr/chungbuk/allim/allimList.json</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>SSL 인증서 오류 — verify=False 필요</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="5" t="inlineStr"/>
-      <c r="B50" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>전주정보문화산업진흥원</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>https://www.jica.or.kr/2025/inner.php?sMenu=A4000</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="inlineStr">
-        <is>
-          <t>SSL 오류 + URL /2016/→/2025/ 변경</t>
-        </is>
-      </c>
+          <t>POST JSON API</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="28" customHeight="1">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>✅ 구현 완료 — 한국예탁결제원 JSON API (1개)</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="n"/>
+      <c r="C50" s="10" t="n"/>
+      <c r="D50" s="10" t="n"/>
+      <c r="E50" s="10" t="n"/>
     </row>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="5" t="inlineStr"/>
@@ -1595,25 +1580,25 @@
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>https://www.ksd.or.kr/ko/about-ksd/ksd-news/bid-notice</t>
+          <t>https://www.ksd.or.kr/ko/api/content?menuId=KR_ABT_070300</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>React SPA — headless browser 필요</t>
+          <t>React SPA → JSON API 직접 호출</t>
         </is>
       </c>
     </row>
     <row r="52" ht="28" customHeight="1">
-      <c r="A52" s="13" t="inlineStr">
+      <c r="A52" s="11" t="inlineStr">
         <is>
           <t>🔄 URL 변경 필요 (1개)</t>
         </is>
       </c>
-      <c r="B52" s="14" t="n"/>
-      <c r="C52" s="14" t="n"/>
-      <c r="D52" s="14" t="n"/>
-      <c r="E52" s="14" t="n"/>
+      <c r="B52" s="12" t="n"/>
+      <c r="C52" s="12" t="n"/>
+      <c r="D52" s="12" t="n"/>
+      <c r="E52" s="12" t="n"/>
     </row>
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="5" t="inlineStr"/>
@@ -1637,15 +1622,15 @@
       </c>
     </row>
     <row r="54" ht="28" customHeight="1">
-      <c r="A54" s="15" t="inlineStr">
+      <c r="A54" s="13" t="inlineStr">
         <is>
           <t>🔧 JS 렌더링 보류 (1개)</t>
         </is>
       </c>
-      <c r="B54" s="16" t="n"/>
-      <c r="C54" s="16" t="n"/>
-      <c r="D54" s="16" t="n"/>
-      <c r="E54" s="16" t="n"/>
+      <c r="B54" s="14" t="n"/>
+      <c r="C54" s="14" t="n"/>
+      <c r="D54" s="14" t="n"/>
+      <c r="E54" s="14" t="n"/>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="5" t="inlineStr"/>
@@ -1669,15 +1654,15 @@
       </c>
     </row>
     <row r="56" ht="28" customHeight="1">
-      <c r="A56" s="17" t="inlineStr">
+      <c r="A56" s="15" t="inlineStr">
         <is>
           <t>❌ 제외 (1개)</t>
         </is>
       </c>
-      <c r="B56" s="18" t="n"/>
-      <c r="C56" s="18" t="n"/>
-      <c r="D56" s="18" t="n"/>
-      <c r="E56" s="18" t="n"/>
+      <c r="B56" s="16" t="n"/>
+      <c r="C56" s="16" t="n"/>
+      <c r="D56" s="16" t="n"/>
+      <c r="E56" s="16" t="n"/>
     </row>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="5" t="inlineStr"/>
@@ -1701,20 +1686,20 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="19" t="inlineStr">
-        <is>
-          <t>※ 구현 완료 43개 사이트는 일괄 수집 버튼 1개로 수집 가능</t>
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>※ 구현 완료 46개 사이트는 일괄 수집 버튼 1개로 수집 가능</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A50:E50"/>
     <mergeCell ref="A59:E59"/>
-    <mergeCell ref="A48:E48"/>
     <mergeCell ref="A54:E54"/>
     <mergeCell ref="A52:E52"/>
+    <mergeCell ref="A42:E42"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A40:E40"/>
     <mergeCell ref="A56:E56"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
@@ -1755,15 +1740,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId48"/>

</xml_diff>

<commit_message>
Phase A.3: 한국지식재산보호원 추가 — 총 47개 사이트 (HTML 39 + CCEI 7 + KSD 1)
한국지식재산보호원 재검증 결과 일반 HTML 테이블로 확인 (JS 렌더링 아님).
JS 렌더링 보류 0개, 추가 조치 필요 0개로 해소.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/work_log2/site_verification.xlsx
+++ b/work_log2/site_verification.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,12 +66,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00375623"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="009C0006"/>
       <sz val="11"/>
     </font>
@@ -82,7 +76,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -107,11 +101,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCD5B4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -146,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -176,11 +165,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -546,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -593,7 +578,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>✅ 구현 완료 — HTML 스크래핑 (38개)</t>
+          <t>✅ 구현 완료 — HTML 스크래핑 (39개)</t>
         </is>
       </c>
       <c r="B3" s="4" t="n"/>
@@ -1399,37 +1384,37 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="28" customHeight="1">
-      <c r="A42" s="9" t="inlineStr">
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="5" t="inlineStr"/>
+      <c r="B42" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>한국지식재산보호원</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>https://www.koipa.re.kr/home/board/brdList.do?menu_cd=000042</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>일반 HTML 테이블 (JS 렌더링 아님)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>✅ 구현 완료 — CCEI 입찰공고 JSON API (7개)</t>
         </is>
       </c>
-      <c r="B42" s="10" t="n"/>
-      <c r="C42" s="10" t="n"/>
-      <c r="D42" s="10" t="n"/>
-      <c r="E42" s="10" t="n"/>
-    </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="5" t="inlineStr"/>
-      <c r="B43" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>CCEI-경기</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>https://ccei.creativekorea.or.kr/gyeonggi/allim/allimList.json</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="inlineStr">
-        <is>
-          <t>POST JSON API</t>
-        </is>
-      </c>
+      <c r="B43" s="10" t="n"/>
+      <c r="C43" s="10" t="n"/>
+      <c r="D43" s="10" t="n"/>
+      <c r="E43" s="10" t="n"/>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="5" t="inlineStr"/>
@@ -1438,12 +1423,12 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>CCEI-경남</t>
+          <t>CCEI-경기</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/gyeongnam/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/gyeonggi/allim/allimList.json</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
@@ -1459,12 +1444,12 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>CCEI-대구</t>
+          <t>CCEI-경남</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/daegu/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/gyeongnam/allim/allimList.json</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -1480,12 +1465,12 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>CCEI-부산</t>
+          <t>CCEI-대구</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/busan/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/daegu/allim/allimList.json</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -1501,12 +1486,12 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>CCEI-세종</t>
+          <t>CCEI-부산</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/sejong/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/busan/allim/allimList.json</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
@@ -1522,12 +1507,12 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>CCEI-인천</t>
+          <t>CCEI-세종</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>https://ccei.creativekorea.or.kr/incheon/allim/allimList.json</t>
+          <t>https://ccei.creativekorea.or.kr/sejong/allim/allimList.json</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -1543,164 +1528,152 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
+          <t>CCEI-인천</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>https://ccei.creativekorea.or.kr/incheon/allim/allimList.json</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>POST JSON API</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="5" t="inlineStr"/>
+      <c r="B50" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
           <t>CCEI-충북</t>
         </is>
       </c>
-      <c r="D49" s="8" t="inlineStr">
+      <c r="D50" s="8" t="inlineStr">
         <is>
           <t>https://ccei.creativekorea.or.kr/chungbuk/allim/allimList.json</t>
         </is>
       </c>
-      <c r="E49" s="7" t="inlineStr">
+      <c r="E50" s="7" t="inlineStr">
         <is>
           <t>POST JSON API</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="28" customHeight="1">
-      <c r="A50" s="9" t="inlineStr">
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
         <is>
           <t>✅ 구현 완료 — 한국예탁결제원 JSON API (1개)</t>
         </is>
       </c>
-      <c r="B50" s="10" t="n"/>
-      <c r="C50" s="10" t="n"/>
-      <c r="D50" s="10" t="n"/>
-      <c r="E50" s="10" t="n"/>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="5" t="inlineStr"/>
-      <c r="B51" s="6" t="n">
-        <v>46</v>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="B51" s="10" t="n"/>
+      <c r="C51" s="10" t="n"/>
+      <c r="D51" s="10" t="n"/>
+      <c r="E51" s="10" t="n"/>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="5" t="inlineStr"/>
+      <c r="B52" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>한국예탁결제원</t>
         </is>
       </c>
-      <c r="D51" s="8" t="inlineStr">
+      <c r="D52" s="8" t="inlineStr">
         <is>
           <t>https://www.ksd.or.kr/ko/api/content?menuId=KR_ABT_070300</t>
         </is>
       </c>
-      <c r="E51" s="7" t="inlineStr">
+      <c r="E52" s="7" t="inlineStr">
         <is>
           <t>React SPA → JSON API 직접 호출</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="28" customHeight="1">
-      <c r="A52" s="11" t="inlineStr">
+    <row r="53" ht="28" customHeight="1">
+      <c r="A53" s="11" t="inlineStr">
         <is>
           <t>🔄 URL 변경 필요 (1개)</t>
         </is>
       </c>
-      <c r="B52" s="12" t="n"/>
-      <c r="C52" s="12" t="n"/>
-      <c r="D52" s="12" t="n"/>
-      <c r="E52" s="12" t="n"/>
-    </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="5" t="inlineStr"/>
-      <c r="B53" s="6" t="n">
-        <v>47</v>
-      </c>
-      <c r="C53" s="7" t="inlineStr">
+      <c r="B53" s="12" t="n"/>
+      <c r="C53" s="12" t="n"/>
+      <c r="D53" s="12" t="n"/>
+      <c r="E53" s="12" t="n"/>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="5" t="inlineStr"/>
+      <c r="B54" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
         <is>
           <t>소상공인시장진흥공단</t>
         </is>
       </c>
-      <c r="D53" s="8" t="inlineStr">
+      <c r="D54" s="8" t="inlineStr">
         <is>
           <t>https://semas.or.kr/web/board/webBoardList.kmdc?bCd=220&amp;pNm=BOA0102</t>
         </is>
       </c>
-      <c r="E53" s="7" t="inlineStr">
+      <c r="E54" s="7" t="inlineStr">
         <is>
           <t>입찰정보 5건뿐, 실효성 낮음</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="28" customHeight="1">
-      <c r="A54" s="13" t="inlineStr">
-        <is>
-          <t>🔧 JS 렌더링 보류 (1개)</t>
-        </is>
-      </c>
-      <c r="B54" s="14" t="n"/>
-      <c r="C54" s="14" t="n"/>
-      <c r="D54" s="14" t="n"/>
-      <c r="E54" s="14" t="n"/>
-    </row>
-    <row r="55" ht="22" customHeight="1">
-      <c r="A55" s="5" t="inlineStr"/>
-      <c r="B55" s="6" t="n">
-        <v>48</v>
-      </c>
-      <c r="C55" s="7" t="inlineStr">
-        <is>
-          <t>한국지식재산보호원</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>https://www.koipa.re.kr/home/board/brdList.do?menu_cd=000042</t>
-        </is>
-      </c>
-      <c r="E55" s="7" t="inlineStr">
-        <is>
-          <t>JS 렌더링 — BeautifulSoup 불가, API 또는 Selenium 필요</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="28" customHeight="1">
-      <c r="A56" s="15" t="inlineStr">
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="13" t="inlineStr">
         <is>
           <t>❌ 제외 (1개)</t>
         </is>
       </c>
-      <c r="B56" s="16" t="n"/>
-      <c r="C56" s="16" t="n"/>
-      <c r="D56" s="16" t="n"/>
-      <c r="E56" s="16" t="n"/>
-    </row>
-    <row r="57" ht="22" customHeight="1">
-      <c r="A57" s="5" t="inlineStr"/>
-      <c r="B57" s="6" t="n">
+      <c r="B55" s="14" t="n"/>
+      <c r="C55" s="14" t="n"/>
+      <c r="D55" s="14" t="n"/>
+      <c r="E55" s="14" t="n"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="5" t="inlineStr"/>
+      <c r="B56" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="C57" s="7" t="inlineStr">
+      <c r="C56" s="7" t="inlineStr">
         <is>
           <t>부산창업포탈</t>
         </is>
       </c>
-      <c r="D57" s="8" t="inlineStr">
+      <c r="D56" s="8" t="inlineStr">
         <is>
           <t>https://busanstartup.kr/biz_sup?mcode=biz02&amp;deleteYn=N&amp;busi_code=820</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr">
+      <c r="E56" s="7" t="inlineStr">
         <is>
           <t>창업지원 프로그램, 입찰 아님</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="17" t="inlineStr">
-        <is>
-          <t>※ 구현 완료 46개 사이트는 일괄 수집 버튼 1개로 수집 가능</t>
+    <row r="58">
+      <c r="A58" s="15" t="inlineStr">
+        <is>
+          <t>※ 구현 완료 47개 사이트는 일괄 수집 버튼 1개로 수집 가능</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="A59:E59"/>
-    <mergeCell ref="A54:E54"/>
-    <mergeCell ref="A52:E52"/>
-    <mergeCell ref="A42:E42"/>
+  <mergeCells count="7">
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A51:E51"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A58:E58"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <hyperlinks>
@@ -1742,17 +1715,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Phase A.3: 부산창업포탈 추가 — 총 48개 사이트 (HTML 39 + CCEI 7 + JSON 2)
부산창업포탈 JSON API (/_Api/bizListData) 직접 호출로 구현.
scrape_busan_startup() 전용 함수 추가. 제외 사이트 0개로 해소.
50개 대상 중 48개 구현, 1개 실효성 낮음(소상공인), 1개 미대응 없음.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/work_log2/site_verification.xlsx
+++ b/work_log2/site_verification.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,18 +65,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="009C0006"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <i val="1"/>
       <color rgb="00666666"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -101,11 +95,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCD5B4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -135,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -161,11 +150,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -531,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1566,7 +1551,7 @@
     <row r="51" ht="28" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>✅ 구현 완료 — 한국예탁결제원 JSON API (1개)</t>
+          <t>✅ 구현 완료 — JSON API (2개)</t>
         </is>
       </c>
       <c r="B51" s="10" t="n"/>
@@ -1595,85 +1580,73 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="28" customHeight="1">
-      <c r="A53" s="11" t="inlineStr">
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="5" t="inlineStr"/>
+      <c r="B53" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>부산창업포탈</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>https://busanstartup.kr/_Api/bizListData</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>JS 렌더링 → JSON API 직접 호출</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="28" customHeight="1">
+      <c r="A54" s="11" t="inlineStr">
         <is>
           <t>🔄 URL 변경 필요 (1개)</t>
         </is>
       </c>
-      <c r="B53" s="12" t="n"/>
-      <c r="C53" s="12" t="n"/>
-      <c r="D53" s="12" t="n"/>
-      <c r="E53" s="12" t="n"/>
-    </row>
-    <row r="54" ht="22" customHeight="1">
-      <c r="A54" s="5" t="inlineStr"/>
-      <c r="B54" s="6" t="n">
+      <c r="B54" s="12" t="n"/>
+      <c r="C54" s="12" t="n"/>
+      <c r="D54" s="12" t="n"/>
+      <c r="E54" s="12" t="n"/>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="5" t="inlineStr"/>
+      <c r="B55" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="C54" s="7" t="inlineStr">
+      <c r="C55" s="7" t="inlineStr">
         <is>
           <t>소상공인시장진흥공단</t>
         </is>
       </c>
-      <c r="D54" s="8" t="inlineStr">
+      <c r="D55" s="8" t="inlineStr">
         <is>
           <t>https://semas.or.kr/web/board/webBoardList.kmdc?bCd=220&amp;pNm=BOA0102</t>
         </is>
       </c>
-      <c r="E54" s="7" t="inlineStr">
+      <c r="E55" s="7" t="inlineStr">
         <is>
           <t>입찰정보 5건뿐, 실효성 낮음</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="28" customHeight="1">
-      <c r="A55" s="13" t="inlineStr">
-        <is>
-          <t>❌ 제외 (1개)</t>
-        </is>
-      </c>
-      <c r="B55" s="14" t="n"/>
-      <c r="C55" s="14" t="n"/>
-      <c r="D55" s="14" t="n"/>
-      <c r="E55" s="14" t="n"/>
-    </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="5" t="inlineStr"/>
-      <c r="B56" s="6" t="n">
-        <v>49</v>
-      </c>
-      <c r="C56" s="7" t="inlineStr">
-        <is>
-          <t>부산창업포탈</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>https://busanstartup.kr/biz_sup?mcode=biz02&amp;deleteYn=N&amp;busi_code=820</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="inlineStr">
-        <is>
-          <t>창업지원 프로그램, 입찰 아님</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="15" t="inlineStr">
-        <is>
-          <t>※ 구현 완료 47개 사이트는 일괄 수집 버튼 1개로 수집 가능</t>
+    <row r="57">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>※ 구현 완료 48개 사이트는 일괄 수집 버튼 1개로 수집 가능 (소상공인시장진흥공단 제외 — 실효성 낮음)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="A55:E55"/>
+  <mergeCells count="6">
     <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A54:E54"/>
     <mergeCell ref="A51:E51"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A58:E58"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <hyperlinks>
@@ -1724,8 +1697,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>